<commit_message>
Added reusable Allure utility methods and test updates
</commit_message>
<xml_diff>
--- a/MyBooking/data/login_data.xlsx
+++ b/MyBooking/data/login_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ukeya\Automation\MyBooking\MyBooking\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\Mybooking\MyBooking\MyBooking\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34C89195-4FD2-4ABE-AC90-69B65F7C7BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{789F3868-E5CC-4BF6-8535-210894C67851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="16210" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -53,12 +53,6 @@
     <t>success</t>
   </si>
   <si>
-    <t>SETCSARYUK</t>
-  </si>
-  <si>
-    <t>mybooking</t>
-  </si>
-  <si>
     <t>minPallets</t>
   </si>
   <si>
@@ -80,27 +74,18 @@
     <t>Incoming Check</t>
   </si>
   <si>
-    <t>Testing Arya</t>
-  </si>
-  <si>
     <t>Consolidate Duplicates</t>
   </si>
   <si>
     <t>Sweden</t>
   </si>
   <si>
-    <t>Testing Edit Arya</t>
-  </si>
-  <si>
     <t>Denmark</t>
   </si>
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>arya.ukey@posten.no</t>
-  </si>
-  <si>
     <t>Title</t>
   </si>
   <si>
@@ -117,6 +102,21 @@
   </si>
   <si>
     <t>AR MyBooking</t>
+  </si>
+  <si>
+    <t>Testing Automation</t>
+  </si>
+  <si>
+    <t>Testing AutomationEditOption</t>
+  </si>
+  <si>
+    <t>SETCSSENN1</t>
+  </si>
+  <si>
+    <t>sweden</t>
+  </si>
+  <si>
+    <t>senna.kamatchi.prabhakar@posten.no</t>
   </si>
 </sst>
 </file>
@@ -537,42 +537,42 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" t="s">
-        <v>11</v>
-      </c>
       <c r="J1" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
@@ -587,25 +587,25 @@
         <v>74601</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="K2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="L2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="M2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
@@ -619,13 +619,13 @@
         <v>2650</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>